<commit_message>
Rebalance stage six and seven pacing and AI research return
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/ai_tech_tree.xlsx
+++ b/space-battleship/config_excel/ai_tech_tree.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ai_tech_tree" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ai_tech_tree" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -504,6 +504,11 @@
           <t>requirements</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>legacy_unlock</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="33" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -556,6 +561,11 @@
           <t>前置：ID:等级;ID:等级</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Legacy research visibility gate</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="33" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -608,6 +618,11 @@
           <t>固定级或 10*k+1</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="40" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -631,7 +646,7 @@
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>1.8</v>
@@ -646,6 +661,11 @@
       </c>
       <c r="I4" s="3" t="inlineStr"/>
       <c r="J4" s="3" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>超时空炼铁炉</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -684,6 +704,11 @@
       </c>
       <c r="I5" s="3" t="inlineStr"/>
       <c r="J5" s="3" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>正电子聚焦装置</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -707,7 +732,7 @@
         </is>
       </c>
       <c r="E6" s="3" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>1.4</v>
@@ -722,6 +747,11 @@
       </c>
       <c r="I6" s="3" t="inlineStr"/>
       <c r="J6" s="3" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>简并态装甲</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -760,6 +790,11 @@
       </c>
       <c r="I7" s="3" t="inlineStr"/>
       <c r="J7" s="3" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>超时空炼铁炉</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="40" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -802,6 +837,11 @@
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>宝石熔炼炉</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="3" t="inlineStr">

</xml_diff>